<commit_message>
fix: align wildberries import with real export layout
</commit_message>
<xml_diff>
--- a/backend-nest/test/fixtures/wb-products-sample.xlsx
+++ b/backend-nest/test/fixtures/wb-products-sample.xlsx
@@ -4,6 +4,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Товары" sheetId="1" r:id="rId1"/>
+    <sheet name="Инструкция" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -397,8 +398,120 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A3:W8"/>
+  <dimension ref="A1:AD7"/>
+  <cols>
+    <col min="1" max="1"/>
+    <col min="2" max="2"/>
+    <col min="3" max="3"/>
+    <col min="4" max="4"/>
+    <col min="5" max="5"/>
+    <col min="6" max="6"/>
+    <col min="7" max="7"/>
+    <col min="8" max="8"/>
+    <col min="9" max="9"/>
+    <col min="10" max="10"/>
+    <col min="11" max="11"/>
+    <col min="12" max="12"/>
+    <col min="13" max="13"/>
+    <col min="14" max="14" hidden="true"/>
+    <col min="15" max="15"/>
+    <col min="16" max="16"/>
+    <col min="17" max="17"/>
+    <col min="18" max="18"/>
+    <col min="19" max="19"/>
+    <col min="20" max="20"/>
+    <col min="21" max="21"/>
+    <col min="22" max="22"/>
+    <col min="23" max="23"/>
+    <col min="24" max="24"/>
+    <col min="25" max="25"/>
+    <col min="26" max="26"/>
+    <col min="27" max="27"/>
+    <col min="28" max="28"/>
+    <col min="29" max="29"/>
+    <col min="30" max="30"/>
+  </cols>
   <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v/>
+      </c>
+      <c r="B1" t="str">
+        <v/>
+      </c>
+      <c r="C1" t="str">
+        <v>Основная информация</v>
+      </c>
+      <c r="D1" t="str">
+        <v/>
+      </c>
+      <c r="E1" t="str">
+        <v/>
+      </c>
+      <c r="F1" t="str">
+        <v/>
+      </c>
+      <c r="G1" t="str">
+        <v/>
+      </c>
+      <c r="H1" t="str">
+        <v/>
+      </c>
+      <c r="I1" t="str">
+        <v/>
+      </c>
+      <c r="J1" t="str">
+        <v/>
+      </c>
+      <c r="K1" t="str">
+        <v/>
+      </c>
+      <c r="L1" t="str">
+        <v/>
+      </c>
+      <c r="M1" t="str">
+        <v/>
+      </c>
+      <c r="N1" t="str">
+        <v/>
+      </c>
+      <c r="O1" t="str">
+        <v/>
+      </c>
+      <c r="P1" t="str">
+        <v/>
+      </c>
+      <c r="Q1" t="str">
+        <v/>
+      </c>
+      <c r="R1" t="str">
+        <v/>
+      </c>
+      <c r="S1" t="str">
+        <v/>
+      </c>
+      <c r="T1" t="str">
+        <v/>
+      </c>
+      <c r="U1" t="str">
+        <v>Размеры и Баркоды</v>
+      </c>
+      <c r="V1" t="str">
+        <v/>
+      </c>
+      <c r="W1" t="str">
+        <v/>
+      </c>
+      <c r="X1" t="str">
+        <v>Цены</v>
+      </c>
+      <c r="Y1" t="str">
+        <v/>
+      </c>
+      <c r="Z1" t="str">
+        <v>Габариты</v>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" t="str">
         <v>Группа</v>
@@ -434,63 +547,268 @@
         <v>Вес с упаковкой (кг)</v>
       </c>
       <c r="L3" t="str">
+        <v>18+</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Только для ИП и юрлиц</v>
+      </c>
+      <c r="N3" t="str">
+        <v>Количество штук в упаковке</v>
+      </c>
+      <c r="O3" t="str">
+        <v>Минимальное количество штук в заказе</v>
+      </c>
+      <c r="P3" t="str">
+        <v>Подтверждаю, что товар промаркирован</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>Вид меха</v>
+      </c>
+      <c r="R3" t="str">
         <v>Пол</v>
       </c>
-      <c r="M3" t="str">
+      <c r="S3" t="str">
         <v>Состав</v>
       </c>
-      <c r="N3" t="str">
+      <c r="T3" t="str">
         <v>Цвет</v>
       </c>
-      <c r="O3" t="str">
+      <c r="U3" t="str">
         <v>Баркоды</v>
       </c>
-      <c r="P3" t="str">
+      <c r="V3" t="str">
         <v>Размер</v>
       </c>
-      <c r="Q3" t="str">
+      <c r="W3" t="str">
         <v>Рос. размер</v>
       </c>
-      <c r="R3" t="str">
+      <c r="X3" t="str">
         <v>Цена</v>
       </c>
-      <c r="S3" t="str">
+      <c r="Y3" t="str">
         <v>Ставка НДС</v>
       </c>
-      <c r="T3" t="str">
+      <c r="Z3" t="str">
+        <v>Вес товара без упаковки (г)</v>
+      </c>
+      <c r="AA3" t="str">
         <v>Вес товара с упаковкой (г)</v>
       </c>
-      <c r="U3" t="str">
+      <c r="AB3" t="str">
         <v>Высота упаковки</v>
       </c>
-      <c r="V3" t="str">
+      <c r="AC3" t="str">
         <v>Длина упаковки</v>
       </c>
-      <c r="W3" t="str">
+      <c r="AD3" t="str">
         <v>Ширина упаковки</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v/>
+      </c>
+      <c r="B4" t="str">
+        <v>SKU help text</v>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v>Category help text</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v>Photo URLs separated by ;</v>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4" t="str">
+        <v/>
+      </c>
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4" t="str">
+        <v/>
+      </c>
+      <c r="V4" t="str">
+        <v/>
+      </c>
+      <c r="W4" t="str">
+        <v/>
+      </c>
+      <c r="X4" t="str">
+        <v>Price help text</v>
+      </c>
+      <c r="Y4" t="str">
+        <v/>
+      </c>
+      <c r="Z4" t="str">
+        <v/>
+      </c>
+      <c r="AA4" t="str">
+        <v/>
+      </c>
+      <c r="AB4" t="str">
+        <v/>
+      </c>
+      <c r="AC4" t="str">
+        <v/>
+      </c>
+      <c r="AD4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5" t="str">
+        <v>SKU-100</v>
+      </c>
+      <c r="C5" t="str">
+        <v>990000001</v>
+      </c>
+      <c r="D5" t="str">
+        <v>WB Linen Shorts</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Shorts</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Demo Brand</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Sanitized description for product one.</v>
+      </c>
+      <c r="H5" t="str">
+        <v>https://example.com/a1.jpg;https://example.com/a2.jpg</v>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v>Нужен</v>
+      </c>
+      <c r="K5">
+        <v>0.5</v>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
+      <c r="R5" t="str">
+        <v>Женский</v>
+      </c>
+      <c r="S5" t="str">
+        <v>cotton;elastane</v>
+      </c>
+      <c r="T5" t="str">
+        <v>blue</v>
+      </c>
+      <c r="U5" t="str">
+        <v>460000000001;460000000099</v>
+      </c>
+      <c r="V5" t="str">
+        <v>S</v>
+      </c>
+      <c r="W5" t="str">
+        <v>42</v>
+      </c>
+      <c r="X5">
+        <v>1200</v>
+      </c>
+      <c r="Y5" t="str">
+        <v>5</v>
+      </c>
+      <c r="Z5" t="str">
+        <v/>
+      </c>
+      <c r="AA5">
+        <v>500</v>
+      </c>
+      <c r="AB5">
+        <v>5</v>
+      </c>
+      <c r="AC5">
+        <v>30</v>
+      </c>
+      <c r="AD5">
+        <v>30</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="str">
-        <v>O</v>
+      <c r="A6">
+        <v>2</v>
       </c>
       <c r="B6" t="str">
         <v>SKU-100</v>
       </c>
       <c r="C6" t="str">
-        <v>9101001</v>
+        <v>990000001</v>
       </c>
       <c r="D6" t="str">
-        <v>WB Linen Dress</v>
+        <v>WB Linen Shorts</v>
       </c>
       <c r="E6" t="str">
-        <v>Dresses</v>
+        <v>Shorts</v>
       </c>
       <c r="F6" t="str">
         <v>Demo Brand</v>
       </c>
       <c r="G6" t="str">
-        <v>Dress description</v>
+        <v>Sanitized description for product one.</v>
       </c>
       <c r="H6" t="str">
         <v>https://example.com/a1.jpg;https://example.com/a2.jpg</v>
@@ -499,193 +817,186 @@
         <v/>
       </c>
       <c r="J6" t="str">
-        <v>нет</v>
-      </c>
-      <c r="K6" t="str">
-        <v>0.4</v>
+        <v>Нужен</v>
+      </c>
+      <c r="K6">
+        <v>0.5</v>
       </c>
       <c r="L6" t="str">
-        <v>Female</v>
+        <v/>
       </c>
       <c r="M6" t="str">
-        <v>Linen 80%; Cotton 20%</v>
+        <v/>
       </c>
       <c r="N6" t="str">
-        <v>White</v>
+        <v/>
       </c>
       <c r="O6" t="str">
-        <v>460000000001</v>
+        <v/>
       </c>
       <c r="P6" t="str">
-        <v>S</v>
+        <v/>
       </c>
       <c r="Q6" t="str">
-        <v>42</v>
+        <v/>
       </c>
       <c r="R6" t="str">
-        <v>1200</v>
+        <v>Женский</v>
       </c>
       <c r="S6" t="str">
-        <v>20</v>
+        <v>cotton;elastane</v>
       </c>
       <c r="T6" t="str">
-        <v>400</v>
+        <v>blue</v>
       </c>
       <c r="U6" t="str">
-        <v>3</v>
+        <v>460000000002</v>
       </c>
       <c r="V6" t="str">
+        <v>M</v>
+      </c>
+      <c r="W6" t="str">
+        <v>44</v>
+      </c>
+      <c r="X6">
+        <v>1300</v>
+      </c>
+      <c r="Y6" t="str">
+        <v>5</v>
+      </c>
+      <c r="Z6" t="str">
+        <v/>
+      </c>
+      <c r="AA6">
+        <v>500</v>
+      </c>
+      <c r="AB6">
+        <v>5</v>
+      </c>
+      <c r="AC6">
         <v>30</v>
       </c>
-      <c r="W6" t="str">
-        <v>20</v>
+      <c r="AD6">
+        <v>30</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="str">
-        <v>O</v>
+      <c r="A7">
+        <v>3</v>
       </c>
       <c r="B7" t="str">
-        <v>SKU-100</v>
+        <v>SKU-200</v>
       </c>
       <c r="C7" t="str">
-        <v>9101001</v>
+        <v>990000002</v>
       </c>
       <c r="D7" t="str">
-        <v>WB Linen Dress</v>
+        <v>WB Cotton Shirt</v>
       </c>
       <c r="E7" t="str">
-        <v>Dresses</v>
+        <v>Shirts</v>
       </c>
       <c r="F7" t="str">
         <v>Demo Brand</v>
       </c>
       <c r="G7" t="str">
-        <v>Dress description</v>
+        <v>Sanitized description for product two.</v>
       </c>
       <c r="H7" t="str">
-        <v>https://example.com/a1.jpg;https://example.com/a2.jpg</v>
+        <v>https://example.com/b1.jpg</v>
       </c>
       <c r="I7" t="str">
         <v/>
       </c>
       <c r="J7" t="str">
-        <v>нет</v>
-      </c>
-      <c r="K7" t="str">
-        <v>0.4</v>
+        <v>Не нужен</v>
+      </c>
+      <c r="K7">
+        <v>0.25</v>
       </c>
       <c r="L7" t="str">
-        <v>Female</v>
+        <v/>
       </c>
       <c r="M7" t="str">
-        <v>Linen 80%; Cotton 20%</v>
+        <v/>
       </c>
       <c r="N7" t="str">
-        <v>White</v>
+        <v/>
       </c>
       <c r="O7" t="str">
-        <v>460000000002</v>
+        <v/>
       </c>
       <c r="P7" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="Q7" t="str">
-        <v>44</v>
+        <v/>
       </c>
       <c r="R7" t="str">
-        <v>1200</v>
+        <v>Мужский</v>
       </c>
       <c r="S7" t="str">
+        <v>cotton</v>
+      </c>
+      <c r="T7" t="str">
+        <v>white</v>
+      </c>
+      <c r="U7" t="str">
+        <v/>
+      </c>
+      <c r="V7" t="str">
+        <v>L</v>
+      </c>
+      <c r="W7" t="str">
+        <v>50</v>
+      </c>
+      <c r="X7">
+        <v>0</v>
+      </c>
+      <c r="Y7" t="str">
+        <v>5</v>
+      </c>
+      <c r="Z7" t="str">
+        <v/>
+      </c>
+      <c r="AA7">
+        <v>250</v>
+      </c>
+      <c r="AB7">
+        <v>4</v>
+      </c>
+      <c r="AC7">
+        <v>25</v>
+      </c>
+      <c r="AD7">
         <v>20</v>
       </c>
-      <c r="T7" t="str">
-        <v>400</v>
-      </c>
-      <c r="U7" t="str">
-        <v>3</v>
-      </c>
-      <c r="V7" t="str">
-        <v>30</v>
-      </c>
-      <c r="W7" t="str">
-        <v>20</v>
-      </c>
     </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>O</v>
-      </c>
-      <c r="B8" t="str">
-        <v>SKU-200</v>
-      </c>
-      <c r="C8" t="str">
-        <v>9101002</v>
-      </c>
-      <c r="D8" t="str">
-        <v>WB Cotton Top</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Tops</v>
-      </c>
-      <c r="F8" t="str">
-        <v>Demo Brand</v>
-      </c>
-      <c r="G8" t="str">
-        <v>Top description</v>
-      </c>
-      <c r="H8" t="str">
-        <v>https://example.com/b1.jpg</v>
-      </c>
-      <c r="I8" t="str">
-        <v/>
-      </c>
-      <c r="J8" t="str">
-        <v>нет</v>
-      </c>
-      <c r="K8" t="str">
-        <v>0.2</v>
-      </c>
-      <c r="L8" t="str">
-        <v>Female</v>
-      </c>
-      <c r="M8" t="str">
-        <v>Cotton 100%</v>
-      </c>
-      <c r="N8" t="str">
-        <v>Red</v>
-      </c>
-      <c r="O8" t="str">
-        <v>460000000003</v>
-      </c>
-      <c r="P8" t="str">
-        <v>One Size</v>
-      </c>
-      <c r="Q8" t="str">
-        <v>OS</v>
-      </c>
-      <c r="R8" t="str">
-        <v>900</v>
-      </c>
-      <c r="S8" t="str">
-        <v>20</v>
-      </c>
-      <c r="T8" t="str">
-        <v>200</v>
-      </c>
-      <c r="U8" t="str">
-        <v>2</v>
-      </c>
-      <c r="V8" t="str">
-        <v>25</v>
-      </c>
-      <c r="W8" t="str">
-        <v>18</v>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="C1:T1"/>
+    <mergeCell ref="U1:W1"/>
+    <mergeCell ref="X1:Y1"/>
+    <mergeCell ref="Z1:AD1"/>
+  </mergeCells>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:AD7"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Sanitized instruction sheet</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A3:W8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>